<commit_message>
Marcado y desmarcado de leyendas, estado de omitido, acelerografos y pluviometros
</commit_message>
<xml_diff>
--- a/resources/workspace/dataequipos.xlsx
+++ b/resources/workspace/dataequipos.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acelerografo1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acelerografo2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -507,7 +507,7 @@
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>MONITOREO DE ACELERÓGRAFOS - LA ARENA</t>
+          <t>MONITOREO DE ACELERÓGRAFOS - ARACELI 2.0</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Acelerografo1</t>
+          <t>Acelerografo2</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0</v>
+        <v>9126061</v>
       </c>
       <c r="E8" s="1" t="n"/>
     </row>
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>0</v>
+        <v>815342</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>3404</v>
       </c>
       <c r="E9" s="1" t="n"/>
     </row>
@@ -623,34 +623,189 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>01/12/2020</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>0</v>
+        <v>0.9683101851851852</v>
       </c>
       <c r="C12" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
-      </c>
+        <v>896.9</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>15/12/2020</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>0</v>
+        <v>0.8613773148148148</v>
       </c>
       <c r="C13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D13" t="n">
+        <v>696.8</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.4834143518518518</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D14" t="n">
+        <v>650.8</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>0.5524652777777778</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D15" t="n">
+        <v>650.8</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.7098958333333333</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>508.2</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.9868634259259259</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D17" t="n">
+        <v>700.6</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>0.02092592592592592</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>562.7</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.09633101851851852</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>914.8</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.277349537037037</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D20" t="n">
+        <v>563.7</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.4697453703703704</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>421.7</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.4159722222222222</v>
+      </c>
+      <c r="C22" t="n">
         <v>5</v>
       </c>
-      <c r="D13" t="n">
-        <v>1</v>
-      </c>
+      <c r="D22" t="n">
+        <v>210</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>